<commit_message>
Cleaned repo and added docker grid setup
</commit_message>
<xml_diff>
--- a/src/test/resources/excel/TestData.xlsx
+++ b/src/test/resources/excel/TestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016"/>
   </bookViews>
   <sheets>
     <sheet name="RUNMANAGER" sheetId="2" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
   <si>
     <t>firstname</t>
   </si>
@@ -105,12 +105,6 @@
   </si>
   <si>
     <t>3</t>
-  </si>
-  <si>
-    <t>asd</t>
-  </si>
-  <si>
-    <t>no</t>
   </si>
   <si>
     <t>browser</t>
@@ -525,7 +519,7 @@
         <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>29</v>
@@ -541,7 +535,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="2"/>
@@ -559,7 +553,7 @@
         <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -582,7 +576,7 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
         <v>3</v>
@@ -605,7 +599,7 @@
         <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -625,10 +619,10 @@
         <v>25</v>
       </c>
       <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
         <v>31</v>
-      </c>
-      <c r="C4" t="s">
-        <v>33</v>
       </c>
       <c r="D4" t="s">
         <v>26</v>
@@ -641,29 +635,6 @@
       </c>
       <c r="G4" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F5" t="s">
-        <v>5</v>
-      </c>
-      <c r="G5" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>